<commit_message>
AVLO update to start year 2021
</commit_message>
<xml_diff>
--- a/InputData/trans/AVLo/Avg Vehicle Loading.xlsx
+++ b/InputData/trans/AVLo/Avg Vehicle Loading.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="11207"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29530"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/skorpius/Library/CloudStorage/GoogleDrive-ferolea@gmail.com/.shortcut-targets-by-id/1HGdhm3a4YN2IE0FhA2aqI2jKTxxSmLoI/EI.ICM/Material de apoyo/Transporte/AVLo/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Olivia Ashmoore\Documents\EPS_Models by Region\eps-mexico\InputData\trans\AVLo\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9258C8B5-048F-2C46-9A55-DAFF8EBFC45B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BC987199-FE7F-461C-AF47-450A4A9AE2D2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="500" windowWidth="33600" windowHeight="17760" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" firstSheet="6" activeTab="11" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="About" sheetId="1" r:id="rId1"/>
@@ -4463,7 +4463,7 @@
     <xf numFmtId="173" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="113">
+  <cellXfs count="119">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -4665,6 +4665,16 @@
     </xf>
     <xf numFmtId="174" fontId="0" fillId="0" borderId="0" xfId="157" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="173" fontId="51" fillId="39" borderId="0" xfId="157" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="159">
     <cellStyle name="20% - Accent1 2" xfId="2" xr:uid="{00000000-0005-0000-0000-000000000000}"/>
@@ -4792,7 +4802,7 @@
     <cellStyle name="Output 2" xfId="118" xr:uid="{00000000-0005-0000-0000-000076000000}"/>
     <cellStyle name="Parent row" xfId="119" xr:uid="{00000000-0005-0000-0000-000077000000}"/>
     <cellStyle name="Parent row 2" xfId="120" xr:uid="{00000000-0005-0000-0000-000078000000}"/>
-    <cellStyle name="Per cent" xfId="155" builtinId="5"/>
+    <cellStyle name="Percent" xfId="155" builtinId="5"/>
     <cellStyle name="Percent 2" xfId="121" xr:uid="{00000000-0005-0000-0000-000079000000}"/>
     <cellStyle name="Percent 2 2" xfId="122" xr:uid="{00000000-0005-0000-0000-00007A000000}"/>
     <cellStyle name="Percent 3" xfId="123" xr:uid="{00000000-0005-0000-0000-00007B000000}"/>
@@ -5160,10 +5170,10 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:D77"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="11.5" customWidth="1"/>
-    <col min="2" max="2" width="85.1640625" customWidth="1"/>
+    <col min="1" max="1" width="11.42578125" customWidth="1"/>
+    <col min="2" max="2" width="85.140625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:4">
@@ -5212,7 +5222,7 @@
         <v>527</v>
       </c>
     </row>
-    <row r="11" spans="1:4" ht="16">
+    <row r="11" spans="1:4" ht="15.75">
       <c r="B11" t="s">
         <v>497</v>
       </c>
@@ -5509,17 +5519,17 @@
     <tabColor theme="3"/>
   </sheetPr>
   <dimension ref="A1:B7"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="11.83203125" customWidth="1"/>
+    <col min="1" max="1" width="11.85546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" s="1" customFormat="1" ht="32">
+    <row r="1" spans="1:2" s="1" customFormat="1" ht="45">
       <c r="A1" s="16" t="s">
         <v>490</v>
       </c>
       <c r="B1" s="1">
-        <v>2022</v>
+        <v>2020</v>
       </c>
     </row>
     <row r="2" spans="1:2">
@@ -5585,184 +5595,190 @@
   <sheetPr>
     <tabColor theme="3"/>
   </sheetPr>
-  <dimension ref="A1:AW7"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
+  <dimension ref="A1:AY7"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="13.1640625" customWidth="1"/>
-    <col min="2" max="2" width="8.6640625" customWidth="1"/>
+    <col min="1" max="1" width="13.140625" customWidth="1"/>
+    <col min="2" max="4" width="8" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:49" ht="48">
+    <row r="1" spans="1:51" ht="45">
       <c r="A1" s="16" t="s">
         <v>483</v>
       </c>
       <c r="B1" s="5">
+        <v>2021</v>
+      </c>
+      <c r="C1" s="5">
+        <v>2022</v>
+      </c>
+      <c r="D1" s="5">
         <v>2023</v>
       </c>
-      <c r="C1" s="5">
+      <c r="E1" s="5">
         <v>2024</v>
       </c>
-      <c r="D1" s="5">
+      <c r="F1" s="5">
         <v>2025</v>
       </c>
-      <c r="E1" s="5">
+      <c r="G1" s="5">
         <v>2026</v>
       </c>
-      <c r="F1" s="5">
+      <c r="H1" s="5">
         <v>2027</v>
       </c>
-      <c r="G1" s="5">
+      <c r="I1" s="5">
         <v>2028</v>
       </c>
-      <c r="H1" s="5">
+      <c r="J1" s="5">
         <v>2029</v>
       </c>
-      <c r="I1" s="5">
+      <c r="K1" s="5">
         <v>2030</v>
       </c>
-      <c r="J1" s="5">
+      <c r="L1" s="5">
         <v>2031</v>
       </c>
-      <c r="K1" s="5">
+      <c r="M1" s="5">
         <v>2032</v>
       </c>
-      <c r="L1" s="5">
+      <c r="N1" s="5">
         <v>2033</v>
       </c>
-      <c r="M1" s="5">
+      <c r="O1" s="5">
         <v>2034</v>
       </c>
-      <c r="N1" s="5">
+      <c r="P1" s="5">
         <v>2035</v>
       </c>
-      <c r="O1" s="5">
+      <c r="Q1" s="5">
         <v>2036</v>
       </c>
-      <c r="P1" s="5">
+      <c r="R1" s="5">
         <v>2037</v>
       </c>
-      <c r="Q1" s="5">
+      <c r="S1" s="5">
         <v>2038</v>
       </c>
-      <c r="R1" s="5">
+      <c r="T1" s="5">
         <v>2039</v>
       </c>
-      <c r="S1" s="5">
+      <c r="U1" s="5">
         <v>2040</v>
       </c>
-      <c r="T1" s="5">
+      <c r="V1" s="5">
         <v>2041</v>
       </c>
-      <c r="U1" s="5">
+      <c r="W1" s="5">
         <v>2042</v>
       </c>
-      <c r="V1" s="5">
+      <c r="X1" s="5">
         <v>2043</v>
       </c>
-      <c r="W1" s="5">
+      <c r="Y1" s="5">
         <v>2044</v>
       </c>
-      <c r="X1" s="5">
+      <c r="Z1" s="5">
         <v>2045</v>
       </c>
-      <c r="Y1" s="5">
+      <c r="AA1" s="5">
         <v>2046</v>
       </c>
-      <c r="Z1" s="5">
+      <c r="AB1" s="5">
         <v>2047</v>
       </c>
-      <c r="AA1" s="5">
+      <c r="AC1" s="5">
         <v>2048</v>
       </c>
-      <c r="AB1" s="5">
+      <c r="AD1" s="5">
         <v>2049</v>
       </c>
-      <c r="AC1" s="5">
+      <c r="AE1" s="5">
         <v>2050</v>
       </c>
-      <c r="AD1" s="5">
+      <c r="AF1" s="5">
         <v>2051</v>
       </c>
-      <c r="AE1" s="5">
+      <c r="AG1" s="5">
         <v>2052</v>
       </c>
-      <c r="AF1" s="5">
+      <c r="AH1" s="5">
         <v>2053</v>
       </c>
-      <c r="AG1" s="5">
+      <c r="AI1" s="5">
         <v>2054</v>
       </c>
-      <c r="AH1" s="5">
+      <c r="AJ1" s="5">
         <v>2055</v>
       </c>
-      <c r="AI1" s="5">
+      <c r="AK1" s="5">
         <v>2056</v>
       </c>
-      <c r="AJ1" s="5">
+      <c r="AL1" s="5">
         <v>2057</v>
       </c>
-      <c r="AK1" s="5">
+      <c r="AM1" s="5">
         <v>2058</v>
       </c>
-      <c r="AL1" s="5">
+      <c r="AN1" s="5">
         <v>2059</v>
       </c>
-      <c r="AM1" s="5">
+      <c r="AO1" s="5">
         <v>2060</v>
       </c>
-      <c r="AN1" s="5">
+      <c r="AP1" s="5">
         <v>2061</v>
       </c>
-      <c r="AO1" s="5">
+      <c r="AQ1" s="5">
         <v>2062</v>
       </c>
-      <c r="AP1" s="5">
+      <c r="AR1" s="5">
         <v>2063</v>
       </c>
-      <c r="AQ1" s="5">
+      <c r="AS1" s="5">
         <v>2064</v>
       </c>
-      <c r="AR1" s="5">
+      <c r="AT1" s="5">
         <v>2065</v>
       </c>
-      <c r="AS1" s="5">
+      <c r="AU1" s="5">
         <v>2066</v>
       </c>
-      <c r="AT1" s="5">
+      <c r="AV1" s="5">
         <v>2067</v>
       </c>
-      <c r="AU1" s="5">
+      <c r="AW1" s="5">
         <v>2068</v>
       </c>
-      <c r="AV1" s="5">
+      <c r="AX1" s="5">
         <v>2069</v>
       </c>
-      <c r="AW1" s="5">
+      <c r="AY1" s="5">
         <v>2070</v>
       </c>
     </row>
-    <row r="2" spans="1:49">
+    <row r="2" spans="1:51">
       <c r="A2" s="1" t="s">
         <v>484</v>
       </c>
-      <c r="B2" s="7">
+      <c r="B2" s="117">
+        <f>C2</f>
+        <v>1.4</v>
+      </c>
+      <c r="C2" s="117">
+        <f>D2</f>
+        <v>1.4</v>
+      </c>
+      <c r="D2" s="7">
         <f>'Mexico Psgr LDVs, Psgr HDVs'!$B$6</f>
         <v>1.4</v>
       </c>
-      <c r="C2" s="7">
-        <f>$B2</f>
+      <c r="E2" s="7">
+        <f>$D2</f>
         <v>1.4</v>
       </c>
-      <c r="D2" s="7">
-        <f t="shared" ref="D2:AE7" si="0">$B2</f>
-        <v>1.4</v>
-      </c>
-      <c r="E2" s="7">
-        <f t="shared" si="0"/>
-        <v>1.4</v>
-      </c>
       <c r="F2" s="7">
-        <f t="shared" si="0"/>
+        <f t="shared" ref="F2:AG7" si="0">$D2</f>
         <v>1.4</v>
       </c>
       <c r="G2" s="7">
@@ -5866,15 +5882,15 @@
         <v>1.4</v>
       </c>
       <c r="AF2" s="7">
-        <f t="shared" ref="AD2:AV7" si="1">$B2</f>
+        <f t="shared" si="0"/>
         <v>1.4</v>
       </c>
       <c r="AG2" s="7">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>1.4</v>
       </c>
       <c r="AH2" s="7">
-        <f t="shared" si="1"/>
+        <f t="shared" ref="AF2:AX7" si="1">$D2</f>
         <v>1.4</v>
       </c>
       <c r="AI2" s="7">
@@ -5934,88 +5950,96 @@
         <v>1.4</v>
       </c>
       <c r="AW2" s="7">
-        <f t="shared" ref="AW2:AW7" si="2">$B2</f>
+        <f t="shared" si="1"/>
         <v>1.4</v>
       </c>
-    </row>
-    <row r="3" spans="1:49">
+      <c r="AX2" s="7">
+        <f t="shared" si="1"/>
+        <v>1.4</v>
+      </c>
+      <c r="AY2" s="7">
+        <f t="shared" ref="AY2:AY7" si="2">$D2</f>
+        <v>1.4</v>
+      </c>
+    </row>
+    <row r="3" spans="1:51">
       <c r="A3" s="1" t="s">
         <v>485</v>
       </c>
-      <c r="B3" s="9">
+      <c r="B3" s="117">
+        <f t="shared" ref="B3:C7" si="3">C3</f>
+        <v>35.666666666666664</v>
+      </c>
+      <c r="C3" s="117">
+        <f t="shared" si="3"/>
+        <v>35.666666666666664</v>
+      </c>
+      <c r="D3" s="9">
         <f>AVERAGE('Mexico Psgr LDVs, Psgr HDVs'!B8:B9,'Mexico Psgr LDVs, Psgr HDVs'!B11)</f>
         <v>35.666666666666664</v>
       </c>
-      <c r="C3" s="7">
-        <f t="shared" ref="C3:R7" si="3">$B3</f>
+      <c r="E3" s="7">
+        <f t="shared" ref="E3:T7" si="4">$D3</f>
         <v>35.666666666666664</v>
       </c>
-      <c r="D3" s="7">
-        <f t="shared" si="3"/>
+      <c r="F3" s="7">
+        <f t="shared" si="4"/>
         <v>35.666666666666664</v>
       </c>
-      <c r="E3" s="7">
-        <f t="shared" si="3"/>
+      <c r="G3" s="7">
+        <f t="shared" si="4"/>
         <v>35.666666666666664</v>
       </c>
-      <c r="F3" s="7">
-        <f t="shared" si="3"/>
+      <c r="H3" s="7">
+        <f t="shared" si="4"/>
         <v>35.666666666666664</v>
       </c>
-      <c r="G3" s="7">
-        <f t="shared" si="3"/>
+      <c r="I3" s="7">
+        <f t="shared" si="4"/>
         <v>35.666666666666664</v>
       </c>
-      <c r="H3" s="7">
-        <f t="shared" si="3"/>
+      <c r="J3" s="7">
+        <f t="shared" si="4"/>
         <v>35.666666666666664</v>
       </c>
-      <c r="I3" s="7">
-        <f t="shared" si="3"/>
+      <c r="K3" s="7">
+        <f t="shared" si="4"/>
         <v>35.666666666666664</v>
       </c>
-      <c r="J3" s="7">
-        <f t="shared" si="3"/>
+      <c r="L3" s="7">
+        <f t="shared" si="4"/>
         <v>35.666666666666664</v>
       </c>
-      <c r="K3" s="7">
-        <f t="shared" si="3"/>
+      <c r="M3" s="7">
+        <f t="shared" si="4"/>
         <v>35.666666666666664</v>
       </c>
-      <c r="L3" s="7">
-        <f t="shared" si="3"/>
+      <c r="N3" s="7">
+        <f t="shared" si="4"/>
         <v>35.666666666666664</v>
       </c>
-      <c r="M3" s="7">
-        <f t="shared" si="3"/>
+      <c r="O3" s="7">
+        <f t="shared" si="4"/>
         <v>35.666666666666664</v>
       </c>
-      <c r="N3" s="7">
-        <f t="shared" si="3"/>
+      <c r="P3" s="7">
+        <f t="shared" si="4"/>
         <v>35.666666666666664</v>
       </c>
-      <c r="O3" s="7">
-        <f t="shared" si="3"/>
+      <c r="Q3" s="7">
+        <f t="shared" si="4"/>
         <v>35.666666666666664</v>
       </c>
-      <c r="P3" s="7">
-        <f t="shared" si="3"/>
+      <c r="R3" s="7">
+        <f t="shared" si="4"/>
         <v>35.666666666666664</v>
       </c>
-      <c r="Q3" s="7">
-        <f t="shared" si="3"/>
+      <c r="S3" s="7">
+        <f t="shared" si="4"/>
         <v>35.666666666666664</v>
       </c>
-      <c r="R3" s="7">
-        <f t="shared" si="3"/>
-        <v>35.666666666666664</v>
-      </c>
-      <c r="S3" s="7">
-        <f t="shared" si="0"/>
-        <v>35.666666666666664</v>
-      </c>
       <c r="T3" s="7">
-        <f t="shared" si="0"/>
+        <f t="shared" si="4"/>
         <v>35.666666666666664</v>
       </c>
       <c r="U3" s="7">
@@ -6055,11 +6079,11 @@
         <v>35.666666666666664</v>
       </c>
       <c r="AD3" s="7">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>35.666666666666664</v>
       </c>
       <c r="AE3" s="7">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>35.666666666666664</v>
       </c>
       <c r="AF3" s="7">
@@ -6131,28 +6155,36 @@
         <v>35.666666666666664</v>
       </c>
       <c r="AW3" s="7">
+        <f t="shared" si="1"/>
+        <v>35.666666666666664</v>
+      </c>
+      <c r="AX3" s="7">
+        <f t="shared" si="1"/>
+        <v>35.666666666666664</v>
+      </c>
+      <c r="AY3" s="7">
         <f t="shared" si="2"/>
         <v>35.666666666666664</v>
       </c>
     </row>
-    <row r="4" spans="1:49">
+    <row r="4" spans="1:51">
       <c r="A4" s="1" t="s">
         <v>486</v>
       </c>
-      <c r="B4" s="9">
+      <c r="B4" s="117">
+        <f t="shared" si="3"/>
+        <v>111.39416306433705</v>
+      </c>
+      <c r="C4" s="117">
+        <f t="shared" si="3"/>
+        <v>111.39416306433705</v>
+      </c>
+      <c r="D4" s="9">
         <f>'BTS NTS Modal Profile Data'!B8</f>
         <v>111.39416306433705</v>
       </c>
-      <c r="C4" s="7">
-        <f t="shared" si="3"/>
-        <v>111.39416306433705</v>
-      </c>
-      <c r="D4" s="7">
-        <f t="shared" si="0"/>
-        <v>111.39416306433705</v>
-      </c>
       <c r="E4" s="7">
-        <f t="shared" si="0"/>
+        <f t="shared" si="4"/>
         <v>111.39416306433705</v>
       </c>
       <c r="F4" s="7">
@@ -6252,11 +6284,11 @@
         <v>111.39416306433705</v>
       </c>
       <c r="AD4" s="7">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>111.39416306433705</v>
       </c>
       <c r="AE4" s="7">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>111.39416306433705</v>
       </c>
       <c r="AF4" s="7">
@@ -6328,28 +6360,36 @@
         <v>111.39416306433705</v>
       </c>
       <c r="AW4" s="7">
+        <f t="shared" si="1"/>
+        <v>111.39416306433705</v>
+      </c>
+      <c r="AX4" s="7">
+        <f t="shared" si="1"/>
+        <v>111.39416306433705</v>
+      </c>
+      <c r="AY4" s="7">
         <f t="shared" si="2"/>
         <v>111.39416306433705</v>
       </c>
     </row>
-    <row r="5" spans="1:49">
+    <row r="5" spans="1:51">
       <c r="A5" s="1" t="s">
         <v>487</v>
       </c>
-      <c r="B5" s="9">
+      <c r="B5" s="117">
+        <f t="shared" si="3"/>
+        <v>15.34784042981183</v>
+      </c>
+      <c r="C5" s="117">
+        <f t="shared" si="3"/>
+        <v>15.34784042981183</v>
+      </c>
+      <c r="D5" s="9">
         <f>'psgr rail calcs'!L62</f>
         <v>15.34784042981183</v>
       </c>
-      <c r="C5" s="7">
-        <f t="shared" si="3"/>
-        <v>15.34784042981183</v>
-      </c>
-      <c r="D5" s="7">
-        <f t="shared" si="0"/>
-        <v>15.34784042981183</v>
-      </c>
       <c r="E5" s="7">
-        <f t="shared" si="0"/>
+        <f t="shared" si="4"/>
         <v>15.34784042981183</v>
       </c>
       <c r="F5" s="7">
@@ -6449,11 +6489,11 @@
         <v>15.34784042981183</v>
       </c>
       <c r="AD5" s="7">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>15.34784042981183</v>
       </c>
       <c r="AE5" s="7">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>15.34784042981183</v>
       </c>
       <c r="AF5" s="7">
@@ -6525,27 +6565,35 @@
         <v>15.34784042981183</v>
       </c>
       <c r="AW5" s="7">
+        <f t="shared" si="1"/>
+        <v>15.34784042981183</v>
+      </c>
+      <c r="AX5" s="7">
+        <f t="shared" si="1"/>
+        <v>15.34784042981183</v>
+      </c>
+      <c r="AY5" s="7">
         <f t="shared" si="2"/>
         <v>15.34784042981183</v>
       </c>
     </row>
-    <row r="6" spans="1:49">
+    <row r="6" spans="1:51">
       <c r="A6" s="1" t="s">
         <v>488</v>
       </c>
-      <c r="B6" s="7">
-        <v>1</v>
-      </c>
-      <c r="C6" s="7">
+      <c r="B6" s="117">
         <f t="shared" si="3"/>
         <v>1</v>
       </c>
+      <c r="C6" s="117">
+        <f t="shared" si="3"/>
+        <v>1</v>
+      </c>
       <c r="D6" s="7">
-        <f t="shared" si="0"/>
         <v>1</v>
       </c>
       <c r="E6" s="7">
-        <f t="shared" si="0"/>
+        <f t="shared" si="4"/>
         <v>1</v>
       </c>
       <c r="F6" s="7">
@@ -6645,11 +6693,11 @@
         <v>1</v>
       </c>
       <c r="AD6" s="7">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>1</v>
       </c>
       <c r="AE6" s="7">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>1</v>
       </c>
       <c r="AF6" s="7">
@@ -6721,28 +6769,36 @@
         <v>1</v>
       </c>
       <c r="AW6" s="7">
+        <f t="shared" si="1"/>
+        <v>1</v>
+      </c>
+      <c r="AX6" s="7">
+        <f t="shared" si="1"/>
+        <v>1</v>
+      </c>
+      <c r="AY6" s="7">
         <f t="shared" si="2"/>
         <v>1</v>
       </c>
     </row>
-    <row r="7" spans="1:49">
+    <row r="7" spans="1:51">
       <c r="A7" s="1" t="s">
         <v>489</v>
       </c>
-      <c r="B7" s="7">
+      <c r="B7" s="117">
+        <f t="shared" si="3"/>
+        <v>1.33</v>
+      </c>
+      <c r="C7" s="117">
+        <f t="shared" si="3"/>
+        <v>1.33</v>
+      </c>
+      <c r="D7" s="7">
         <f>'Mexico Psgr LDVs, Psgr HDVs'!B15</f>
         <v>1.33</v>
       </c>
-      <c r="C7" s="7">
-        <f t="shared" si="3"/>
-        <v>1.33</v>
-      </c>
-      <c r="D7" s="7">
-        <f t="shared" si="0"/>
-        <v>1.33</v>
-      </c>
       <c r="E7" s="7">
-        <f t="shared" si="0"/>
+        <f t="shared" si="4"/>
         <v>1.33</v>
       </c>
       <c r="F7" s="7">
@@ -6842,11 +6898,11 @@
         <v>1.33</v>
       </c>
       <c r="AD7" s="7">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>1.33</v>
       </c>
       <c r="AE7" s="7">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>1.33</v>
       </c>
       <c r="AF7" s="7">
@@ -6918,6 +6974,14 @@
         <v>1.33</v>
       </c>
       <c r="AW7" s="7">
+        <f t="shared" si="1"/>
+        <v>1.33</v>
+      </c>
+      <c r="AX7" s="7">
+        <f t="shared" si="1"/>
+        <v>1.33</v>
+      </c>
+      <c r="AY7" s="7">
         <f t="shared" si="2"/>
         <v>1.33</v>
       </c>
@@ -6932,178 +6996,184 @@
   <sheetPr>
     <tabColor theme="3"/>
   </sheetPr>
-  <dimension ref="A1:AX7"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
+  <dimension ref="A1:AZ7"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="11.83203125" customWidth="1"/>
+    <col min="1" max="3" width="11.85546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:50" s="1" customFormat="1" ht="32">
+    <row r="1" spans="1:52" s="1" customFormat="1" ht="45">
       <c r="A1" s="16" t="s">
         <v>490</v>
       </c>
-      <c r="B1" s="1">
+      <c r="B1" s="16">
+        <v>2021</v>
+      </c>
+      <c r="C1" s="16">
+        <v>2022</v>
+      </c>
+      <c r="D1" s="1">
         <v>2023</v>
       </c>
-      <c r="C1" s="1">
+      <c r="E1" s="1">
         <v>2024</v>
       </c>
-      <c r="D1" s="1">
+      <c r="F1" s="1">
         <v>2025</v>
       </c>
-      <c r="E1" s="1">
+      <c r="G1" s="1">
         <v>2026</v>
       </c>
-      <c r="F1" s="1">
+      <c r="H1" s="1">
         <v>2027</v>
       </c>
-      <c r="G1" s="1">
+      <c r="I1" s="1">
         <v>2028</v>
       </c>
-      <c r="H1" s="1">
+      <c r="J1" s="1">
         <v>2029</v>
       </c>
-      <c r="I1" s="1">
+      <c r="K1" s="1">
         <v>2030</v>
       </c>
-      <c r="J1" s="1">
+      <c r="L1" s="1">
         <v>2031</v>
       </c>
-      <c r="K1" s="1">
+      <c r="M1" s="1">
         <v>2032</v>
       </c>
-      <c r="L1" s="1">
+      <c r="N1" s="1">
         <v>2033</v>
       </c>
-      <c r="M1" s="1">
+      <c r="O1" s="1">
         <v>2034</v>
       </c>
-      <c r="N1" s="1">
+      <c r="P1" s="1">
         <v>2035</v>
       </c>
-      <c r="O1" s="1">
+      <c r="Q1" s="1">
         <v>2036</v>
       </c>
-      <c r="P1" s="1">
+      <c r="R1" s="1">
         <v>2037</v>
       </c>
-      <c r="Q1" s="1">
+      <c r="S1" s="1">
         <v>2038</v>
       </c>
-      <c r="R1" s="1">
+      <c r="T1" s="1">
         <v>2039</v>
       </c>
-      <c r="S1" s="1">
+      <c r="U1" s="1">
         <v>2040</v>
       </c>
-      <c r="T1" s="1">
+      <c r="V1" s="1">
         <v>2041</v>
       </c>
-      <c r="U1" s="1">
+      <c r="W1" s="1">
         <v>2042</v>
       </c>
-      <c r="V1" s="1">
+      <c r="X1" s="1">
         <v>2043</v>
       </c>
-      <c r="W1" s="1">
+      <c r="Y1" s="1">
         <v>2044</v>
       </c>
-      <c r="X1" s="1">
+      <c r="Z1" s="1">
         <v>2045</v>
       </c>
-      <c r="Y1" s="1">
+      <c r="AA1" s="1">
         <v>2046</v>
       </c>
-      <c r="Z1" s="1">
+      <c r="AB1" s="1">
         <v>2047</v>
       </c>
-      <c r="AA1" s="1">
+      <c r="AC1" s="1">
         <v>2048</v>
       </c>
-      <c r="AB1" s="1">
+      <c r="AD1" s="1">
         <v>2049</v>
       </c>
-      <c r="AC1" s="1">
+      <c r="AE1" s="1">
         <v>2050</v>
       </c>
-      <c r="AD1" s="1">
+      <c r="AF1" s="1">
         <v>2051</v>
       </c>
-      <c r="AE1" s="1">
+      <c r="AG1" s="1">
         <v>2052</v>
       </c>
-      <c r="AF1" s="1">
+      <c r="AH1" s="1">
         <v>2053</v>
       </c>
-      <c r="AG1" s="1">
+      <c r="AI1" s="1">
         <v>2054</v>
       </c>
-      <c r="AH1" s="1">
+      <c r="AJ1" s="1">
         <v>2055</v>
       </c>
-      <c r="AI1" s="1">
+      <c r="AK1" s="1">
         <v>2056</v>
       </c>
-      <c r="AJ1" s="1">
+      <c r="AL1" s="1">
         <v>2057</v>
       </c>
-      <c r="AK1" s="1">
+      <c r="AM1" s="1">
         <v>2058</v>
       </c>
-      <c r="AL1" s="1">
+      <c r="AN1" s="1">
         <v>2059</v>
       </c>
-      <c r="AM1" s="1">
+      <c r="AO1" s="1">
         <v>2060</v>
       </c>
-      <c r="AN1" s="1">
+      <c r="AP1" s="1">
         <v>2061</v>
       </c>
-      <c r="AO1" s="1">
+      <c r="AQ1" s="1">
         <v>2062</v>
       </c>
-      <c r="AP1" s="1">
+      <c r="AR1" s="1">
         <v>2063</v>
       </c>
-      <c r="AQ1" s="1">
+      <c r="AS1" s="1">
         <v>2064</v>
       </c>
-      <c r="AR1" s="1">
+      <c r="AT1" s="1">
         <v>2065</v>
       </c>
-      <c r="AS1" s="1">
+      <c r="AU1" s="1">
         <v>2066</v>
       </c>
-      <c r="AT1" s="1">
+      <c r="AV1" s="1">
         <v>2067</v>
       </c>
-      <c r="AU1" s="1">
+      <c r="AW1" s="1">
         <v>2068</v>
       </c>
-      <c r="AV1" s="1">
+      <c r="AX1" s="1">
         <v>2069</v>
       </c>
-      <c r="AW1" s="1">
+      <c r="AY1" s="1">
         <v>2070</v>
       </c>
     </row>
-    <row r="2" spans="1:50">
+    <row r="2" spans="1:52">
       <c r="A2" s="1" t="s">
         <v>484</v>
       </c>
-      <c r="B2" s="14">
+      <c r="B2" s="118">
+        <f>C2</f>
         <v>1</v>
       </c>
-      <c r="C2">
-        <f t="shared" ref="C2:F7" si="0">$B2</f>
+      <c r="C2" s="118">
+        <f>D2</f>
         <v>1</v>
       </c>
-      <c r="D2">
-        <f t="shared" si="0"/>
+      <c r="D2" s="14">
         <v>1</v>
       </c>
       <c r="E2">
-        <f t="shared" si="0"/>
+        <f t="shared" ref="E2:H7" si="0">$D2</f>
         <v>1</v>
       </c>
       <c r="F2">
@@ -7111,15 +7181,15 @@
         <v>1</v>
       </c>
       <c r="G2">
-        <f t="shared" ref="G2:P7" si="1">$B2</f>
+        <f t="shared" si="0"/>
         <v>1</v>
       </c>
       <c r="H2">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>1</v>
       </c>
       <c r="I2">
-        <f t="shared" si="1"/>
+        <f t="shared" ref="I2:R7" si="1">$D2</f>
         <v>1</v>
       </c>
       <c r="J2">
@@ -7151,15 +7221,15 @@
         <v>1</v>
       </c>
       <c r="Q2">
-        <f t="shared" ref="Q2:AF7" si="2">$B2</f>
+        <f t="shared" si="1"/>
         <v>1</v>
       </c>
       <c r="R2">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>1</v>
       </c>
       <c r="S2">
-        <f t="shared" si="2"/>
+        <f t="shared" ref="S2:AH7" si="2">$D2</f>
         <v>1</v>
       </c>
       <c r="T2">
@@ -7215,15 +7285,15 @@
         <v>1</v>
       </c>
       <c r="AG2">
-        <f t="shared" ref="AD2:AS7" si="3">$B2</f>
+        <f t="shared" si="2"/>
         <v>1</v>
       </c>
       <c r="AH2">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>1</v>
       </c>
       <c r="AI2">
-        <f t="shared" si="3"/>
+        <f t="shared" ref="AF2:AU7" si="3">$D2</f>
         <v>1</v>
       </c>
       <c r="AJ2">
@@ -7267,36 +7337,44 @@
         <v>1</v>
       </c>
       <c r="AT2">
-        <f t="shared" ref="AT2:AX7" si="4">$B2</f>
+        <f t="shared" si="3"/>
         <v>1</v>
       </c>
       <c r="AU2">
-        <f t="shared" si="4"/>
+        <f t="shared" si="3"/>
         <v>1</v>
       </c>
       <c r="AV2">
-        <f t="shared" si="4"/>
+        <f t="shared" ref="AV2:AY7" si="4">$D2</f>
         <v>1</v>
       </c>
       <c r="AW2">
         <f t="shared" si="4"/>
         <v>1</v>
       </c>
-    </row>
-    <row r="3" spans="1:50">
+      <c r="AX2">
+        <f t="shared" si="4"/>
+        <v>1</v>
+      </c>
+      <c r="AY2">
+        <f t="shared" si="4"/>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3" spans="1:52">
       <c r="A3" s="1" t="s">
         <v>485</v>
       </c>
-      <c r="B3" s="6">
+      <c r="B3" s="118">
+        <f t="shared" ref="B3:C7" si="5">C3</f>
+        <v>17.260730580665893</v>
+      </c>
+      <c r="C3" s="118">
+        <f t="shared" si="5"/>
+        <v>17.260730580665893</v>
+      </c>
+      <c r="D3" s="6">
         <f>'Mexico Freight Activity'!$U$19</f>
-        <v>17.260730580665893</v>
-      </c>
-      <c r="C3">
-        <f t="shared" si="0"/>
-        <v>17.260730580665893</v>
-      </c>
-      <c r="D3">
-        <f t="shared" si="0"/>
         <v>17.260730580665893</v>
       </c>
       <c r="E3">
@@ -7308,11 +7386,11 @@
         <v>17.260730580665893</v>
       </c>
       <c r="G3">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>17.260730580665893</v>
       </c>
       <c r="H3">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>17.260730580665893</v>
       </c>
       <c r="I3">
@@ -7348,11 +7426,11 @@
         <v>17.260730580665893</v>
       </c>
       <c r="Q3">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>17.260730580665893</v>
       </c>
       <c r="R3">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>17.260730580665893</v>
       </c>
       <c r="S3">
@@ -7400,11 +7478,11 @@
         <v>17.260730580665893</v>
       </c>
       <c r="AD3">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>17.260730580665893</v>
       </c>
       <c r="AE3">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>17.260730580665893</v>
       </c>
       <c r="AF3">
@@ -7464,11 +7542,11 @@
         <v>17.260730580665893</v>
       </c>
       <c r="AT3">
-        <f t="shared" si="4"/>
+        <f t="shared" si="3"/>
         <v>17.260730580665893</v>
       </c>
       <c r="AU3">
-        <f t="shared" si="4"/>
+        <f t="shared" si="3"/>
         <v>17.260730580665893</v>
       </c>
       <c r="AV3">
@@ -7479,21 +7557,29 @@
         <f t="shared" si="4"/>
         <v>17.260730580665893</v>
       </c>
-    </row>
-    <row r="4" spans="1:50">
+      <c r="AX3">
+        <f t="shared" si="4"/>
+        <v>17.260730580665893</v>
+      </c>
+      <c r="AY3">
+        <f t="shared" si="4"/>
+        <v>17.260730580665893</v>
+      </c>
+    </row>
+    <row r="4" spans="1:52">
       <c r="A4" s="1" t="s">
         <v>486</v>
       </c>
-      <c r="B4" s="6">
+      <c r="B4" s="118">
+        <f t="shared" si="5"/>
+        <v>41.989116133258747</v>
+      </c>
+      <c r="C4" s="118">
+        <f t="shared" si="5"/>
+        <v>41.989116133258747</v>
+      </c>
+      <c r="D4" s="6">
         <f>'BTS NTS Modal Profile Data'!B9</f>
-        <v>41.989116133258747</v>
-      </c>
-      <c r="C4" s="6">
-        <f t="shared" si="0"/>
-        <v>41.989116133258747</v>
-      </c>
-      <c r="D4" s="6">
-        <f t="shared" si="0"/>
         <v>41.989116133258747</v>
       </c>
       <c r="E4" s="6">
@@ -7505,11 +7591,11 @@
         <v>41.989116133258747</v>
       </c>
       <c r="G4" s="6">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>41.989116133258747</v>
       </c>
       <c r="H4" s="6">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>41.989116133258747</v>
       </c>
       <c r="I4" s="6">
@@ -7545,11 +7631,11 @@
         <v>41.989116133258747</v>
       </c>
       <c r="Q4" s="6">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>41.989116133258747</v>
       </c>
       <c r="R4" s="6">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>41.989116133258747</v>
       </c>
       <c r="S4" s="6">
@@ -7597,11 +7683,11 @@
         <v>41.989116133258747</v>
       </c>
       <c r="AD4" s="6">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>41.989116133258747</v>
       </c>
       <c r="AE4" s="6">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>41.989116133258747</v>
       </c>
       <c r="AF4" s="6">
@@ -7661,11 +7747,11 @@
         <v>41.989116133258747</v>
       </c>
       <c r="AT4" s="6">
-        <f t="shared" si="4"/>
+        <f t="shared" si="3"/>
         <v>41.989116133258747</v>
       </c>
       <c r="AU4" s="6">
-        <f t="shared" si="4"/>
+        <f t="shared" si="3"/>
         <v>41.989116133258747</v>
       </c>
       <c r="AV4" s="6">
@@ -7676,22 +7762,30 @@
         <f t="shared" si="4"/>
         <v>41.989116133258747</v>
       </c>
-      <c r="AX4" s="6"/>
-    </row>
-    <row r="5" spans="1:50">
+      <c r="AX4" s="6">
+        <f t="shared" si="4"/>
+        <v>41.989116133258747</v>
+      </c>
+      <c r="AY4" s="6">
+        <f t="shared" si="4"/>
+        <v>41.989116133258747</v>
+      </c>
+      <c r="AZ4" s="6"/>
+    </row>
+    <row r="5" spans="1:52">
       <c r="A5" s="1" t="s">
         <v>487</v>
       </c>
-      <c r="B5" s="6">
+      <c r="B5" s="118">
+        <f t="shared" si="5"/>
+        <v>3512.35916421195</v>
+      </c>
+      <c r="C5" s="118">
+        <f t="shared" si="5"/>
+        <v>3512.35916421195</v>
+      </c>
+      <c r="D5" s="6">
         <f>'BTS NTS Modal Profile Data'!B19</f>
-        <v>3512.35916421195</v>
-      </c>
-      <c r="C5" s="6">
-        <f t="shared" si="0"/>
-        <v>3512.35916421195</v>
-      </c>
-      <c r="D5" s="6">
-        <f t="shared" si="0"/>
         <v>3512.35916421195</v>
       </c>
       <c r="E5" s="6">
@@ -7703,11 +7797,11 @@
         <v>3512.35916421195</v>
       </c>
       <c r="G5" s="6">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>3512.35916421195</v>
       </c>
       <c r="H5" s="6">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>3512.35916421195</v>
       </c>
       <c r="I5" s="6">
@@ -7743,11 +7837,11 @@
         <v>3512.35916421195</v>
       </c>
       <c r="Q5" s="6">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>3512.35916421195</v>
       </c>
       <c r="R5" s="6">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>3512.35916421195</v>
       </c>
       <c r="S5" s="6">
@@ -7795,11 +7889,11 @@
         <v>3512.35916421195</v>
       </c>
       <c r="AD5" s="6">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>3512.35916421195</v>
       </c>
       <c r="AE5" s="6">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>3512.35916421195</v>
       </c>
       <c r="AF5" s="6">
@@ -7859,11 +7953,11 @@
         <v>3512.35916421195</v>
       </c>
       <c r="AT5" s="6">
-        <f t="shared" si="4"/>
+        <f t="shared" si="3"/>
         <v>3512.35916421195</v>
       </c>
       <c r="AU5" s="6">
-        <f t="shared" si="4"/>
+        <f t="shared" si="3"/>
         <v>3512.35916421195</v>
       </c>
       <c r="AV5" s="6">
@@ -7874,22 +7968,30 @@
         <f t="shared" si="4"/>
         <v>3512.35916421195</v>
       </c>
-      <c r="AX5" s="6"/>
-    </row>
-    <row r="6" spans="1:50">
+      <c r="AX5" s="6">
+        <f t="shared" si="4"/>
+        <v>3512.35916421195</v>
+      </c>
+      <c r="AY5" s="6">
+        <f t="shared" si="4"/>
+        <v>3512.35916421195</v>
+      </c>
+      <c r="AZ5" s="6"/>
+    </row>
+    <row r="6" spans="1:52">
       <c r="A6" s="1" t="s">
         <v>488</v>
       </c>
-      <c r="B6" s="6">
+      <c r="B6" s="118">
+        <f t="shared" si="5"/>
+        <v>1974.4736422180429</v>
+      </c>
+      <c r="C6" s="118">
+        <f t="shared" si="5"/>
+        <v>1974.4736422180429</v>
+      </c>
+      <c r="D6" s="6">
         <f>'BTS NTS Modal Profile Data'!B55</f>
-        <v>1974.4736422180429</v>
-      </c>
-      <c r="C6" s="6">
-        <f t="shared" si="0"/>
-        <v>1974.4736422180429</v>
-      </c>
-      <c r="D6" s="6">
-        <f t="shared" si="0"/>
         <v>1974.4736422180429</v>
       </c>
       <c r="E6" s="6">
@@ -7901,11 +8003,11 @@
         <v>1974.4736422180429</v>
       </c>
       <c r="G6" s="6">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>1974.4736422180429</v>
       </c>
       <c r="H6" s="6">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>1974.4736422180429</v>
       </c>
       <c r="I6" s="6">
@@ -7941,11 +8043,11 @@
         <v>1974.4736422180429</v>
       </c>
       <c r="Q6" s="6">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>1974.4736422180429</v>
       </c>
       <c r="R6" s="6">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>1974.4736422180429</v>
       </c>
       <c r="S6" s="6">
@@ -7993,11 +8095,11 @@
         <v>1974.4736422180429</v>
       </c>
       <c r="AD6" s="6">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>1974.4736422180429</v>
       </c>
       <c r="AE6" s="6">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>1974.4736422180429</v>
       </c>
       <c r="AF6" s="6">
@@ -8057,11 +8159,11 @@
         <v>1974.4736422180429</v>
       </c>
       <c r="AT6" s="6">
-        <f t="shared" si="4"/>
+        <f t="shared" si="3"/>
         <v>1974.4736422180429</v>
       </c>
       <c r="AU6" s="6">
-        <f t="shared" si="4"/>
+        <f t="shared" si="3"/>
         <v>1974.4736422180429</v>
       </c>
       <c r="AV6" s="6">
@@ -8072,21 +8174,29 @@
         <f t="shared" si="4"/>
         <v>1974.4736422180429</v>
       </c>
-      <c r="AX6" s="6"/>
-    </row>
-    <row r="7" spans="1:50">
+      <c r="AX6" s="6">
+        <f t="shared" si="4"/>
+        <v>1974.4736422180429</v>
+      </c>
+      <c r="AY6" s="6">
+        <f t="shared" si="4"/>
+        <v>1974.4736422180429</v>
+      </c>
+      <c r="AZ6" s="6"/>
+    </row>
+    <row r="7" spans="1:52">
       <c r="A7" s="1" t="s">
         <v>489</v>
       </c>
-      <c r="B7">
-        <v>0</v>
-      </c>
-      <c r="C7">
-        <f t="shared" si="0"/>
+      <c r="B7" s="118">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+      <c r="C7" s="118">
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
       <c r="D7">
-        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="E7">
@@ -8098,11 +8208,11 @@
         <v>0</v>
       </c>
       <c r="G7">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="H7">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="I7">
@@ -8138,11 +8248,11 @@
         <v>0</v>
       </c>
       <c r="Q7">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="R7">
-        <f t="shared" si="2"/>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="S7">
@@ -8190,11 +8300,11 @@
         <v>0</v>
       </c>
       <c r="AD7">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="AE7">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="AF7">
@@ -8254,11 +8364,11 @@
         <v>0</v>
       </c>
       <c r="AT7">
-        <f t="shared" si="4"/>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="AU7">
-        <f t="shared" si="4"/>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="AV7">
@@ -8266,6 +8376,14 @@
         <v>0</v>
       </c>
       <c r="AW7">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="AX7">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="AY7">
         <f t="shared" si="4"/>
         <v>0</v>
       </c>
@@ -8279,11 +8397,11 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:C69"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="73.5" customWidth="1"/>
+    <col min="1" max="1" width="73.42578125" customWidth="1"/>
     <col min="2" max="2" width="12" customWidth="1"/>
-    <col min="3" max="3" width="102.33203125" customWidth="1"/>
+    <col min="3" max="3" width="102.28515625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3">
@@ -8563,7 +8681,7 @@
         <v>33.023738872403563</v>
       </c>
     </row>
-    <row r="37" spans="1:3" ht="16">
+    <row r="37" spans="1:3">
       <c r="A37" s="10" t="s">
         <v>74</v>
       </c>
@@ -8734,7 +8852,7 @@
         <v>17287</v>
       </c>
     </row>
-    <row r="60" spans="1:2" ht="16">
+    <row r="60" spans="1:2">
       <c r="A60" s="10" t="s">
         <v>95</v>
       </c>
@@ -8800,16 +8918,16 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BD61947A-6C1C-43CC-935A-F2AA06F299CA}">
   <dimension ref="A1:AX71"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15"/>
   <cols>
-    <col min="14" max="14" width="9.1640625" style="37"/>
+    <col min="14" max="14" width="9.140625" style="37"/>
     <col min="15" max="23" width="0" hidden="1" customWidth="1"/>
-    <col min="24" max="24" width="11.5" style="37" customWidth="1"/>
+    <col min="24" max="24" width="11.42578125" style="37" customWidth="1"/>
     <col min="25" max="45" width="0" hidden="1" customWidth="1"/>
-    <col min="46" max="46" width="13.5" style="37" customWidth="1"/>
+    <col min="46" max="46" width="13.42578125" style="37" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:50" ht="73">
+    <row r="1" spans="1:50" ht="79.5">
       <c r="A1" s="17" t="s">
         <v>101</v>
       </c>
@@ -16843,17 +16961,17 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2C7BE35E-A64A-47AA-8B99-250F6A5F2C34}">
   <dimension ref="A1:BG70"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15"/>
   <cols>
-    <col min="12" max="12" width="11.33203125" customWidth="1"/>
-    <col min="13" max="13" width="11.1640625" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="11.6640625" customWidth="1"/>
-    <col min="25" max="25" width="12.6640625" customWidth="1"/>
-    <col min="29" max="29" width="11.1640625" customWidth="1"/>
-    <col min="40" max="40" width="11.1640625" customWidth="1"/>
+    <col min="12" max="12" width="11.28515625" customWidth="1"/>
+    <col min="13" max="13" width="11.140625" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="11.7109375" customWidth="1"/>
+    <col min="25" max="25" width="12.7109375" customWidth="1"/>
+    <col min="29" max="29" width="11.140625" customWidth="1"/>
+    <col min="40" max="40" width="11.140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:59" ht="73">
+    <row r="1" spans="1:59" ht="90.75">
       <c r="A1" s="38" t="s">
         <v>101</v>
       </c>
@@ -24964,23 +25082,23 @@
     <tabColor rgb="FFFFCC66"/>
   </sheetPr>
   <dimension ref="B2:X64"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15"/>
   <cols>
-    <col min="2" max="2" width="18.33203125" customWidth="1"/>
-    <col min="3" max="3" width="9.83203125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="11.5" customWidth="1"/>
-    <col min="5" max="5" width="22.5" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="15.33203125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="16.83203125" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="15.83203125" customWidth="1"/>
-    <col min="9" max="9" width="18.5" customWidth="1"/>
-    <col min="10" max="10" width="16.5" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="17.83203125" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="9.6640625" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="14.33203125" bestFit="1" customWidth="1"/>
-    <col min="14" max="20" width="14.33203125" customWidth="1"/>
-    <col min="21" max="21" width="18.1640625" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="19.5" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="18.28515625" customWidth="1"/>
+    <col min="3" max="3" width="9.85546875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="11.42578125" customWidth="1"/>
+    <col min="5" max="5" width="22.42578125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="15.28515625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="16.85546875" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="15.85546875" customWidth="1"/>
+    <col min="9" max="9" width="18.42578125" customWidth="1"/>
+    <col min="10" max="10" width="16.42578125" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="17.85546875" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="9.7109375" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="14.28515625" bestFit="1" customWidth="1"/>
+    <col min="14" max="20" width="14.28515625" customWidth="1"/>
+    <col min="21" max="21" width="18.140625" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="19.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="2" spans="2:22">
@@ -29497,12 +29615,12 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{712B411F-69F6-F74D-82DA-9D553D211C18}">
   <dimension ref="A1:B17"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="10.83203125" defaultRowHeight="15"/>
+  <sheetFormatPr defaultColWidth="10.85546875" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="2" width="22.5" style="10" customWidth="1"/>
+    <col min="1" max="2" width="22.42578125" style="10" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" ht="48">
+    <row r="1" spans="1:2" ht="45">
       <c r="A1" s="81" t="s">
         <v>508</v>
       </c>
@@ -29510,7 +29628,7 @@
         <v>509</v>
       </c>
     </row>
-    <row r="2" spans="1:2" ht="32">
+    <row r="2" spans="1:2" ht="45">
       <c r="A2" s="82" t="s">
         <v>510</v>
       </c>
@@ -29518,7 +29636,7 @@
         <v>511</v>
       </c>
     </row>
-    <row r="3" spans="1:2" ht="16">
+    <row r="3" spans="1:2">
       <c r="A3" s="83" t="s">
         <v>512</v>
       </c>
@@ -29526,7 +29644,7 @@
         <v>513</v>
       </c>
     </row>
-    <row r="4" spans="1:2" ht="16">
+    <row r="4" spans="1:2">
       <c r="A4" s="84"/>
       <c r="B4" s="84" t="s">
         <v>514</v>
@@ -29538,7 +29656,7 @@
       </c>
       <c r="B5" s="86"/>
     </row>
-    <row r="6" spans="1:2" ht="14.5" customHeight="1">
+    <row r="6" spans="1:2" ht="14.45" customHeight="1">
       <c r="A6" s="87" t="s">
         <v>516</v>
       </c>
@@ -29631,9 +29749,9 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B6B50426-665B-CD4A-A393-E653E41CDD72}">
   <dimension ref="A1:O30"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11.6640625" defaultRowHeight="16"/>
+  <sheetFormatPr defaultColWidth="11.7109375" defaultRowHeight="15.75"/>
   <cols>
-    <col min="1" max="16384" width="11.6640625" style="90"/>
+    <col min="1" max="16384" width="11.7109375" style="90"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:15">
@@ -29651,7 +29769,7 @@
         <v>529</v>
       </c>
     </row>
-    <row r="5" spans="1:15" ht="17">
+    <row r="5" spans="1:15" ht="16.5">
       <c r="B5" s="92" t="s">
         <v>530</v>
       </c>
@@ -29744,30 +29862,30 @@
         <v>390</v>
       </c>
     </row>
-    <row r="10" spans="1:15" ht="17">
+    <row r="10" spans="1:15" ht="16.5">
       <c r="B10" s="92" t="s">
         <v>536</v>
       </c>
     </row>
-    <row r="13" spans="1:15" ht="17">
+    <row r="13" spans="1:15" ht="16.5">
       <c r="B13" s="92" t="s">
         <v>537</v>
       </c>
     </row>
-    <row r="14" spans="1:15" ht="17">
+    <row r="14" spans="1:15" ht="16.5">
       <c r="B14" s="92" t="s">
         <v>538</v>
       </c>
     </row>
-    <row r="16" spans="1:15" ht="17">
+    <row r="16" spans="1:15" ht="16.5">
       <c r="B16" s="95"/>
     </row>
-    <row r="18" spans="1:5" ht="17">
+    <row r="18" spans="1:5" ht="16.5">
       <c r="B18" s="95" t="s">
         <v>539</v>
       </c>
     </row>
-    <row r="19" spans="1:5" ht="17">
+    <row r="19" spans="1:5" ht="16.5">
       <c r="B19" s="96"/>
     </row>
     <row r="20" spans="1:5">
@@ -29856,11 +29974,11 @@
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C0401F08-C5F4-3843-9CCC-99969C1303FC}">
   <dimension ref="A1:X24"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="10.83203125" defaultRowHeight="15"/>
+  <sheetFormatPr defaultColWidth="10.85546875" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="24" customWidth="1"/>
     <col min="2" max="16" width="0" hidden="1" customWidth="1"/>
-    <col min="21" max="21" width="11.1640625" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="11.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:22" ht="15" customHeight="1">
@@ -30570,74 +30688,80 @@
   <sheetPr>
     <tabColor theme="3"/>
   </sheetPr>
-  <dimension ref="A1:D7"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
+  <dimension ref="A1:C7"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="13.1640625" customWidth="1"/>
-    <col min="2" max="2" width="8.6640625" customWidth="1"/>
+    <col min="1" max="1" width="13.140625" style="115" customWidth="1"/>
+    <col min="2" max="2" width="8.7109375" style="115" customWidth="1"/>
+    <col min="3" max="16384" width="8.85546875" style="115"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" ht="48">
-      <c r="A1" s="16" t="s">
+    <row r="1" spans="1:3" ht="45">
+      <c r="A1" s="113" t="s">
         <v>483</v>
       </c>
-      <c r="B1" s="5">
-        <v>2022</v>
-      </c>
-    </row>
-    <row r="2" spans="1:4">
-      <c r="A2" s="1" t="s">
+      <c r="B1" s="114">
+        <v>2020</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3">
+      <c r="A2" s="116" t="s">
         <v>484</v>
       </c>
-      <c r="B2" s="7">
+      <c r="B2" s="115">
         <f>'Mexico Psgr LDVs, Psgr HDVs'!$B$6</f>
         <v>1.4</v>
       </c>
-    </row>
-    <row r="3" spans="1:4">
-      <c r="A3" s="1" t="s">
+      <c r="C2" s="7"/>
+    </row>
+    <row r="3" spans="1:3">
+      <c r="A3" s="116" t="s">
         <v>485</v>
       </c>
-      <c r="B3" s="9">
+      <c r="B3" s="115">
         <f>AVERAGE('Mexico Psgr LDVs, Psgr HDVs'!B8:B9,'Mexico Psgr LDVs, Psgr HDVs'!B11)</f>
         <v>35.666666666666664</v>
       </c>
-    </row>
-    <row r="4" spans="1:4">
-      <c r="A4" s="1" t="s">
+      <c r="C3" s="7"/>
+    </row>
+    <row r="4" spans="1:3">
+      <c r="A4" s="116" t="s">
         <v>486</v>
       </c>
-      <c r="B4" s="9">
+      <c r="B4" s="115">
         <f>'BTS NTS Modal Profile Data'!B8</f>
         <v>111.39416306433705</v>
       </c>
-    </row>
-    <row r="5" spans="1:4">
-      <c r="A5" s="1" t="s">
+      <c r="C4" s="7"/>
+    </row>
+    <row r="5" spans="1:3">
+      <c r="A5" s="116" t="s">
         <v>487</v>
       </c>
-      <c r="B5" s="9">
+      <c r="B5" s="115">
         <f>'psgr rail calcs'!L62</f>
         <v>15.34784042981183</v>
       </c>
-    </row>
-    <row r="6" spans="1:4">
-      <c r="A6" s="1" t="s">
+      <c r="C5" s="7"/>
+    </row>
+    <row r="6" spans="1:3">
+      <c r="A6" s="116" t="s">
         <v>488</v>
       </c>
-      <c r="B6" s="7">
+      <c r="B6" s="115">
         <v>1</v>
       </c>
-    </row>
-    <row r="7" spans="1:4">
-      <c r="A7" s="1" t="s">
+      <c r="C6" s="7"/>
+    </row>
+    <row r="7" spans="1:3">
+      <c r="A7" s="116" t="s">
         <v>489</v>
       </c>
-      <c r="B7" s="7">
+      <c r="B7" s="115">
         <f>'Mexico Psgr LDVs, Psgr HDVs'!B15</f>
         <v>1.33</v>
       </c>
-      <c r="D7" s="7"/>
+      <c r="C7" s="7"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -30645,18 +30769,18 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
   <Display>DocumentLibraryForm</Display>
   <Edit>DocumentLibraryForm</Edit>
   <New>DocumentLibraryForm</New>
 </FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
@@ -30804,14 +30928,6 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F5F9B18E-AA43-4321-AB68-0D427F1586FD}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9EC57927-87FD-4D66-8290-F178F4C3B3CA}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
@@ -30820,6 +30936,28 @@
 </ds:datastoreItem>
 </file>
 
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F5F9B18E-AA43-4321-AB68-0D427F1586FD}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7DAD2C54-C1B3-40B5-9981-4AC53E268479}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7DAD2C54-C1B3-40B5-9981-4AC53E268479}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="79748b23-d81a-423e-9112-21109dc864e6"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>